<commit_message>
fix: SF8 header rows show their full labels; no stray comment
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/forms/sf8-template.xlsx
+++ b/templates/forms/sf8-template.xlsx
@@ -12,33 +12,6 @@
   <definedNames/>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
 </workbook>
-</file>
-
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author/>
-  </authors>
-  <commentList>
-    <comment ref="A124" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <rFont val="Calibri"/>
-            <b val="false"/>
-            <i val="false"/>
-            <strike val="false"/>
-            <color rgb="FF000000"/>
-            <sz val="11"/>
-            <u val="none"/>
-          </rPr>
-          <t xml:space="preserve">Michael Angelo:
-Date of measurement.</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1971,7 +1944,7 @@
       <c r="N8" s="2"/>
       <c r="O8" s="2"/>
     </row>
-    <row r="9" spans="1:15" customHeight="1" ht="16.5">
+    <row r="9" spans="1:15" customHeight="1" ht="24">
       <c r="A9" s="67" t="s">
         <v>13</v>
       </c>
@@ -2010,7 +1983,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:15" customHeight="1" ht="16.5">
+    <row r="10" spans="1:15" customHeight="1" ht="30">
       <c r="A10" s="68"/>
       <c r="B10" s="78"/>
       <c r="C10" s="74"/>
@@ -5084,6 +5057,5 @@
     <brk id="61" man="1"/>
   </rowBreaks>
   <drawing r:id="rId1"/>
-  <legacyDrawing r:id="rId_comments_vml1"/>
 </worksheet>
 </file>
</xml_diff>